<commit_message>
Sep 5, 2026, 11:11 PM
</commit_message>
<xml_diff>
--- a/reports/swarnim_thakre.xlsx
+++ b/reports/swarnim_thakre.xlsx
@@ -421,22 +421,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,6 +503,73 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>llc1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>06-09-2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>No Lecture</t>
         </is>
       </c>
     </row>
@@ -586,17 +653,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
     </row>
@@ -607,17 +674,17 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
     </row>
@@ -628,17 +695,17 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>77.78%</t>
         </is>
       </c>
     </row>
@@ -712,17 +779,17 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -733,13 +800,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -843,7 +910,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>62.50%</t>
+          <t>62.16%</t>
         </is>
       </c>
     </row>

</xml_diff>